<commit_message>
beta 0.4 - added group division for prettymouth
</commit_message>
<xml_diff>
--- a/excluded.xlsx
+++ b/excluded.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micha\PycharmProjects\wholeBrain_narrative_MAC_MFT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCAEEF07-8D4D-4B28-89B6-07EC2553F145}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71FE593C-1A2C-483F-8C44-E2DF8370EAE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
   <si>
     <t>black</t>
   </si>
@@ -281,6 +281,18 @@
   </si>
   <si>
     <t>139</t>
+  </si>
+  <si>
+    <t>083,084,085,086,032,038,087,034,088,050,089,090,091,092,093,094,095,023,096,097</t>
+  </si>
+  <si>
+    <t>098,065,081,099,100,066,079,101,052,102,030,103,104,105,106,107,108,109,110,111</t>
+  </si>
+  <si>
+    <t>prettymouthaffair</t>
+  </si>
+  <si>
+    <t>prettymouthparanoia</t>
   </si>
 </sst>
 </file>
@@ -328,8 +340,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -632,7 +645,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="40.85546875" customWidth="1"/>
@@ -743,6 +756,22 @@
         <v>4</v>
       </c>
     </row>
+    <row r="16" spans="1:2">
+      <c r="A16" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
beta 0.4 - added whole prettymouth analysis and sherlock
</commit_message>
<xml_diff>
--- a/excluded.xlsx
+++ b/excluded.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micha\PycharmProjects\wholeBrain_narrative_MAC_MFT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71FE593C-1A2C-483F-8C44-E2DF8370EAE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9507299-9B57-42A0-BEBA-298692EDC278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
   <si>
     <t>black</t>
   </si>
@@ -293,6 +293,9 @@
   </si>
   <si>
     <t>prettymouthparanoia</t>
+  </si>
+  <si>
+    <t>prettymouth</t>
   </si>
 </sst>
 </file>
@@ -645,7 +648,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="40.85546875" customWidth="1"/>
@@ -772,6 +775,11 @@
         <v>25</v>
       </c>
     </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
beta 1.1 - update with new sentence parsing and moving files for unused stories to backup folders
</commit_message>
<xml_diff>
--- a/excluded.xlsx
+++ b/excluded.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micha\PycharmProjects\wholeBrain_narrative_MAC_MFT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF93C036-E29E-4737-9E43-25FC08C5CDEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C30FA6ED-7EE5-4B4F-AE2C-D5D1A9A9E885}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -772,7 +772,7 @@
       <c r="A13" t="s">
         <v>21</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="1" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>